<commit_message>
Mapa: Bass 6 y Cluza en construcción junto al canal (sin precio; pin muestra En obra)
</commit_message>
<xml_diff>
--- a/Propiedades.xlsx
+++ b/Propiedades.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -607,7 +607,6 @@
       <c r="G2" t="n">
         <v>1250000</v>
       </c>
-      <c r="H2" t="inlineStr"/>
       <c r="I2" t="inlineStr">
         <is>
           <t>3 + 1 (sótano)</t>
@@ -748,7 +747,6 @@
           <t>Centris 9134776</t>
         </is>
       </c>
-      <c r="T3" t="inlineStr"/>
       <c r="U3" t="inlineStr">
         <is>
           <t>https://www.centris.ca/fr/maison~a-vendre~laval-laval-ouest/9134776</t>
@@ -795,7 +793,6 @@
       <c r="G4" t="n">
         <v>998000</v>
       </c>
-      <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
           <t>4 (1 en sótano)</t>
@@ -835,7 +832,6 @@
           <t>Centris 21686888</t>
         </is>
       </c>
-      <c r="T4" t="inlineStr"/>
       <c r="U4" t="inlineStr">
         <is>
           <t>https://www.centris.ca/fr/maison~a-vendre~laval-sainte-rose/21686888?nocontext=true</t>
@@ -985,7 +981,6 @@
       <c r="G6" t="n">
         <v>769999</v>
       </c>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
           <t>4</t>
@@ -1028,7 +1023,6 @@
           <t>DuProprio #973877</t>
         </is>
       </c>
-      <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/laval/ste-rose/maison-a-vendre/hab-1255-rue-armand-auclair-973877</t>
@@ -1075,7 +1069,6 @@
       <c r="G7" t="n">
         <v>849000</v>
       </c>
-      <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
           <t>4</t>
@@ -1118,7 +1111,6 @@
           <t>DuProprio #742986</t>
         </is>
       </c>
-      <c r="T7" t="inlineStr"/>
       <c r="U7" t="inlineStr">
         <is>
           <t>https://duproprio.com/fr/laval/laval-ouest/maison-a-vendre/hab-6825-rue-monnier-742986</t>
@@ -1165,7 +1157,6 @@
       <c r="G8" t="n">
         <v>699999</v>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
           <t>1</t>
@@ -1223,6 +1214,142 @@
       <c r="W8" t="inlineStr">
         <is>
           <t>Borde de rivière (rivière des Mille-Îles), plan d'eau navigable. Abrigo para auto (1) + entrada (2). Chimenea a gas. Emménagement 30 días después de la aceptación. Cerca de tren de banlieue y transporte en común.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bass6</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Bass 6 (Îlot D2)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Griffintown, Le Sud-Ouest, Montréal</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Condo</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>45.48776</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-73.56515</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>En construcción</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>Musto (promotor)</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=201%20Rue%20Richmond%2C%20Montr%C3%A9al%2C%20QC</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>Ver en Street View</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>🏗️ En construcción (foto oct 2026). 8 pisos, 160 unidades (48% estudios, 25% 1 rec., 21% 2 rec., 6% 3 rec.). Promotor Musto; planos PIIA aprobados jun 2024. Lote entre Richmond (oeste), des Bassins (norte), parc du Bassin-à-Bois (este) y canal (sur). Precios y modalidad (venta/renta) por confirmar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cluza</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Cluza, Appartements sur Bassins</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Griffintown, Le Sud-Ouest, Montréal</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>Condo</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>45.48636</v>
+      </c>
+      <c r="F10" t="n">
+        <v>-73.56722000000001</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>En construcción</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>Omnia Technologies + Claridge (promotores)</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>https://www.google.com/maps/search/?api=1&amp;query=1712%20Rue%20des%20Bassins%2C%20Montr%C3%A9al%2C%20QC</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>Ver en Street View</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>🏗️ En construcción desde 2025, entrega prevista 2027. 9 pisos, 286 unidades. Promotores Omnia Technologies + Claridge. Terreno de las antiguas écuries Lucky Luc. Precios y modalidad (venta/renta) por confirmar. Ubicación del pin aproximada sobre rue des Bassins.</t>
         </is>
       </c>
     </row>
@@ -1250,9 +1377,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -1267,9 +1392,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
@@ -1319,9 +1442,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" t="inlineStr"/>
-    </row>
+    <row r="13"/>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>

</xml_diff>